<commit_message>
Repeat run 2 reproducibly (seed set for each DGM)
</commit_message>
<xml_diff>
--- a/simrun_results_run2.xlsx
+++ b/simrun_results_run2.xlsx
@@ -445,25 +445,25 @@
         <v>5000</v>
       </c>
       <c r="C3">
+        <v>0.0238</v>
+      </c>
+      <c r="D3">
+        <v>0.0258</v>
+      </c>
+      <c r="E3">
+        <v>0.0294</v>
+      </c>
+      <c r="F3">
         <v>0.0232</v>
       </c>
-      <c r="D3">
-        <v>0.024</v>
-      </c>
-      <c r="E3">
-        <v>0.026</v>
-      </c>
-      <c r="F3">
-        <v>0.026</v>
-      </c>
       <c r="G3">
-        <v>0.0216</v>
+        <v>0.0218</v>
       </c>
       <c r="H3">
-        <v>0.0254</v>
+        <v>0.0248</v>
       </c>
       <c r="I3">
-        <v>0.136</v>
+        <v>0.1388</v>
       </c>
     </row>
     <row r="4">
@@ -474,25 +474,25 @@
         <v>5000</v>
       </c>
       <c r="C4">
-        <v>0.0106</v>
+        <v>0.0126</v>
       </c>
       <c r="D4">
         <v>0.0018</v>
       </c>
       <c r="E4">
-        <v>0.0148</v>
+        <v>0.0118</v>
       </c>
       <c r="F4">
-        <v>0.0092</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="G4">
-        <v>0.003</v>
+        <v>0.0026</v>
       </c>
       <c r="H4">
         <v>0.0024</v>
       </c>
       <c r="I4">
-        <v>0.031</v>
+        <v>0.0296</v>
       </c>
     </row>
     <row r="5">
@@ -529,31 +529,31 @@
         <v>5000</v>
       </c>
       <c r="C6">
-        <v>0.6048</v>
+        <v>0.6056</v>
       </c>
       <c r="D6">
-        <v>0.1608</v>
+        <v>0.1492</v>
       </c>
       <c r="E6">
-        <v>0.6556</v>
+        <v>0.6568000000000001</v>
       </c>
       <c r="F6">
-        <v>0.4412</v>
+        <v>0.45</v>
       </c>
       <c r="G6">
-        <v>0.2302</v>
+        <v>0.2352</v>
       </c>
       <c r="H6">
-        <v>0.1722</v>
+        <v>0.1666</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>0.3774666666666667</v>
+        <v>0.3772333333333333</v>
       </c>
       <c r="K6">
-        <v>0.4938608534837486</v>
+        <v>0.4959680683341809</v>
       </c>
     </row>
     <row r="7">
@@ -564,31 +564,31 @@
         <v>5000</v>
       </c>
       <c r="C7">
-        <v>0.8492</v>
+        <v>0.8446</v>
       </c>
       <c r="D7">
-        <v>0.5284</v>
+        <v>0.5154</v>
       </c>
       <c r="E7">
-        <v>0.8672</v>
+        <v>0.8688</v>
       </c>
       <c r="F7">
-        <v>0.76</v>
+        <v>0.7655999999999999</v>
       </c>
       <c r="G7">
-        <v>0.601</v>
+        <v>0.6074000000000001</v>
       </c>
       <c r="H7">
-        <v>0.5392</v>
+        <v>0.5352</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>0.6908333333333333</v>
+        <v>0.6895000000000001</v>
       </c>
       <c r="K7">
-        <v>0.7732419691155393</v>
+        <v>0.7733143187387304</v>
       </c>
     </row>
     <row r="8">
@@ -625,31 +625,31 @@
         <v>5000</v>
       </c>
       <c r="C9">
-        <v>0.7328</v>
+        <v>0.7334000000000001</v>
       </c>
       <c r="D9">
-        <v>0.196</v>
+        <v>0.203</v>
       </c>
       <c r="E9">
-        <v>0.7718</v>
+        <v>0.776</v>
       </c>
       <c r="F9">
-        <v>0.5594</v>
+        <v>0.5698</v>
       </c>
       <c r="G9">
-        <v>0.2928</v>
+        <v>0.2964</v>
       </c>
       <c r="H9">
-        <v>0.2218</v>
+        <v>0.2258</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9">
-        <v>0.4624333333333333</v>
+        <v>0.4674</v>
       </c>
       <c r="K9">
-        <v>0.600376734939202</v>
+        <v>0.6054844075084378</v>
       </c>
     </row>
     <row r="10">
@@ -660,31 +660,31 @@
         <v>5000</v>
       </c>
       <c r="C10">
-        <v>0.9194</v>
+        <v>0.919</v>
       </c>
       <c r="D10">
-        <v>0.63</v>
+        <v>0.634</v>
       </c>
       <c r="E10">
-        <v>0.9330000000000001</v>
+        <v>0.9322</v>
       </c>
       <c r="F10">
-        <v>0.8536</v>
+        <v>0.8612</v>
       </c>
       <c r="G10">
-        <v>0.719</v>
+        <v>0.7098</v>
       </c>
       <c r="H10">
-        <v>0.6566</v>
+        <v>0.6496</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>0.7852666666666667</v>
+        <v>0.7843</v>
       </c>
       <c r="K10">
-        <v>0.8565736326228675</v>
+        <v>0.8575774215174071</v>
       </c>
     </row>
     <row r="11">
@@ -721,31 +721,31 @@
         <v>5000</v>
       </c>
       <c r="C12">
-        <v>0.8276</v>
+        <v>0.8324</v>
       </c>
       <c r="D12">
-        <v>0.2364</v>
+        <v>0.2442</v>
       </c>
       <c r="E12">
-        <v>0.8612</v>
+        <v>0.856</v>
       </c>
       <c r="F12">
-        <v>0.6616</v>
+        <v>0.6636</v>
       </c>
       <c r="G12">
-        <v>0.3582</v>
+        <v>0.3552</v>
       </c>
       <c r="H12">
-        <v>0.2704</v>
+        <v>0.2692</v>
       </c>
       <c r="I12">
         <v>0</v>
       </c>
       <c r="J12">
-        <v>0.5358999999999999</v>
+        <v>0.5367666666666667</v>
       </c>
       <c r="K12">
-        <v>0.6871576702575246</v>
+        <v>0.687745020574229</v>
       </c>
     </row>
     <row r="13">
@@ -756,31 +756,31 @@
         <v>5000</v>
       </c>
       <c r="C13">
-        <v>0.9578</v>
+        <v>0.9592000000000001</v>
       </c>
       <c r="D13">
-        <v>0.7236</v>
+        <v>0.7248</v>
       </c>
       <c r="E13">
-        <v>0.9686</v>
+        <v>0.9678</v>
       </c>
       <c r="F13">
-        <v>0.914</v>
+        <v>0.908</v>
       </c>
       <c r="G13">
-        <v>0.7958</v>
+        <v>0.7822</v>
       </c>
       <c r="H13">
-        <v>0.7452</v>
+        <v>0.7344000000000001</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
       <c r="J13">
-        <v>0.8508333333333334</v>
+        <v>0.8460666666666667</v>
       </c>
       <c r="K13">
-        <v>0.9094465786675298</v>
+        <v>0.9065494683064405</v>
       </c>
     </row>
     <row r="14">
@@ -817,31 +817,31 @@
         <v>5000</v>
       </c>
       <c r="C15">
-        <v>0.8902</v>
+        <v>0.8848</v>
       </c>
       <c r="D15">
-        <v>0.275</v>
+        <v>0.281</v>
       </c>
       <c r="E15">
-        <v>0.9126</v>
+        <v>0.921</v>
       </c>
       <c r="F15">
-        <v>0.7488</v>
+        <v>0.7476</v>
       </c>
       <c r="G15">
-        <v>0.4158</v>
+        <v>0.4064</v>
       </c>
       <c r="H15">
-        <v>0.3072</v>
+        <v>0.318</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
       <c r="J15">
-        <v>0.5916</v>
+        <v>0.5931333333333334</v>
       </c>
       <c r="K15">
-        <v>0.7497344352489712</v>
+        <v>0.7507470410097554</v>
       </c>
     </row>
     <row r="16">
@@ -852,31 +852,31 @@
         <v>5000</v>
       </c>
       <c r="C16">
-        <v>0.9818</v>
+        <v>0.9758</v>
       </c>
       <c r="D16">
-        <v>0.778</v>
+        <v>0.7868000000000001</v>
       </c>
       <c r="E16">
-        <v>0.9816</v>
+        <v>0.9856</v>
       </c>
       <c r="F16">
-        <v>0.9458</v>
+        <v>0.9452</v>
       </c>
       <c r="G16">
-        <v>0.837</v>
+        <v>0.8414</v>
       </c>
       <c r="H16">
-        <v>0.7936</v>
+        <v>0.8028</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
       <c r="J16">
-        <v>0.8863</v>
+        <v>0.8896000000000001</v>
       </c>
       <c r="K16">
-        <v>0.937138887604605</v>
+        <v>0.9380253247954136</v>
       </c>
     </row>
     <row r="17">
@@ -913,31 +913,31 @@
         <v>5000</v>
       </c>
       <c r="C18">
-        <v>0.8296</v>
+        <v>0.8248</v>
       </c>
       <c r="D18">
-        <v>0.2272</v>
+        <v>0.2408</v>
       </c>
       <c r="E18">
-        <v>0.8632</v>
+        <v>0.8612</v>
       </c>
       <c r="F18">
-        <v>0.6606</v>
+        <v>0.6642</v>
       </c>
       <c r="G18">
-        <v>0.3652</v>
+        <v>0.3636</v>
       </c>
       <c r="H18">
-        <v>0.0234</v>
+        <v>0.026</v>
       </c>
       <c r="I18">
-        <v>0.0234</v>
+        <v>0.026</v>
       </c>
       <c r="J18">
-        <v>0.58916</v>
+        <v>0.59092</v>
       </c>
       <c r="K18">
-        <v>0.7097230348083171</v>
+        <v>0.7098162349591814</v>
       </c>
     </row>
     <row r="19">
@@ -948,31 +948,31 @@
         <v>5000</v>
       </c>
       <c r="C19">
-        <v>0.9438</v>
+        <v>0.9412</v>
       </c>
       <c r="D19">
-        <v>0.6128</v>
+        <v>0.6014</v>
       </c>
       <c r="E19">
-        <v>0.954</v>
+        <v>0.9594</v>
       </c>
       <c r="F19">
-        <v>0.875</v>
+        <v>0.8778</v>
       </c>
       <c r="G19">
-        <v>0.7108</v>
+        <v>0.702</v>
       </c>
       <c r="H19">
-        <v>0.2558</v>
+        <v>0.266</v>
       </c>
       <c r="I19">
-        <v>0.2558</v>
+        <v>0.266</v>
       </c>
       <c r="J19">
-        <v>0.81928</v>
+        <v>0.8163600000000001</v>
       </c>
       <c r="K19">
-        <v>0.8839130266567712</v>
+        <v>0.8840634847249766</v>
       </c>
     </row>
     <row r="20">
@@ -1009,31 +1009,31 @@
         <v>5000</v>
       </c>
       <c r="C21">
-        <v>0.8206</v>
+        <v>0.8352000000000001</v>
       </c>
       <c r="D21">
-        <v>0.2408</v>
+        <v>0.2358</v>
       </c>
       <c r="E21">
-        <v>0.0274</v>
+        <v>0.0244</v>
       </c>
       <c r="F21">
-        <v>0.663</v>
+        <v>0.656</v>
       </c>
       <c r="G21">
-        <v>0.3598</v>
+        <v>0.3786</v>
       </c>
       <c r="H21">
-        <v>0.2684</v>
+        <v>0.2712</v>
       </c>
       <c r="I21">
-        <v>0.0274</v>
+        <v>0.0244</v>
       </c>
       <c r="J21">
-        <v>0.47052</v>
+        <v>0.4753600000000001</v>
       </c>
       <c r="K21">
-        <v>0.6169096597323013</v>
+        <v>0.6209825770037091</v>
       </c>
     </row>
     <row r="22">
@@ -1044,31 +1044,31 @@
         <v>5000</v>
       </c>
       <c r="C22">
-        <v>0.9038</v>
+        <v>0.914</v>
       </c>
       <c r="D22">
-        <v>0.4</v>
+        <v>0.3974</v>
       </c>
       <c r="E22">
-        <v>0.1178</v>
+        <v>0.1208</v>
       </c>
       <c r="F22">
-        <v>0.8008</v>
+        <v>0.7966</v>
       </c>
       <c r="G22">
-        <v>0.5362</v>
+        <v>0.5484</v>
       </c>
       <c r="H22">
-        <v>0.4312</v>
+        <v>0.4448</v>
       </c>
       <c r="I22">
-        <v>0.1178</v>
+        <v>0.1208</v>
       </c>
       <c r="J22">
-        <v>0.6144000000000001</v>
+        <v>0.62024</v>
       </c>
       <c r="K22">
-        <v>0.7432542460893404</v>
+        <v>0.7471701144976617</v>
       </c>
     </row>
     <row r="23">
@@ -1105,31 +1105,31 @@
         <v>5000</v>
       </c>
       <c r="C24">
-        <v>0.0258</v>
+        <v>0.022</v>
       </c>
       <c r="D24">
-        <v>0.0284</v>
+        <v>0.026</v>
       </c>
       <c r="E24">
-        <v>0.0234</v>
+        <v>0.0248</v>
       </c>
       <c r="F24">
-        <v>0.0282</v>
+        <v>0.0294</v>
       </c>
       <c r="G24">
-        <v>0.025</v>
+        <v>0.0272</v>
       </c>
       <c r="H24">
-        <v>0.2532</v>
+        <v>0.2616</v>
       </c>
       <c r="I24">
-        <v>0.1244</v>
+        <v>0.1234</v>
       </c>
       <c r="J24">
-        <v>0.2532</v>
+        <v>0.2616</v>
       </c>
       <c r="K24">
-        <v>0.2532</v>
+        <v>0.2616</v>
       </c>
     </row>
     <row r="25">
@@ -1140,31 +1140,31 @@
         <v>5000</v>
       </c>
       <c r="C25">
-        <v>0.0182</v>
+        <v>0.0174</v>
       </c>
       <c r="D25">
-        <v>0.0028</v>
+        <v>0.0036</v>
       </c>
       <c r="E25">
-        <v>0.0204</v>
+        <v>0.0194</v>
       </c>
       <c r="F25">
-        <v>0.0148</v>
+        <v>0.0202</v>
       </c>
       <c r="G25">
-        <v>0.0042</v>
+        <v>0.0068</v>
       </c>
       <c r="H25">
-        <v>0.0318</v>
+        <v>0.0346</v>
       </c>
       <c r="I25">
-        <v>0.049</v>
+        <v>0.0544</v>
       </c>
       <c r="J25">
-        <v>0.0318</v>
+        <v>0.0346</v>
       </c>
       <c r="K25">
-        <v>0.0318</v>
+        <v>0.0346</v>
       </c>
     </row>
     <row r="26">
@@ -1201,31 +1201,31 @@
         <v>5000</v>
       </c>
       <c r="C27">
-        <v>0.0262</v>
+        <v>0.0238</v>
       </c>
       <c r="D27">
-        <v>0.0248</v>
+        <v>0.026</v>
       </c>
       <c r="E27">
-        <v>0.8716</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="F27">
-        <v>0.0294</v>
+        <v>0.0246</v>
       </c>
       <c r="G27">
-        <v>0.0284</v>
+        <v>0.0244</v>
       </c>
       <c r="H27">
-        <v>0.0262</v>
+        <v>0.0264</v>
       </c>
       <c r="I27">
-        <v>0.1282</v>
+        <v>0.118</v>
       </c>
       <c r="J27">
-        <v>0.8716</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="K27">
-        <v>0.8716</v>
+        <v>0.8614000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1236,31 +1236,31 @@
         <v>5000</v>
       </c>
       <c r="C28">
-        <v>0.0374</v>
+        <v>0.0354</v>
       </c>
       <c r="D28">
-        <v>0.012</v>
+        <v>0.0136</v>
       </c>
       <c r="E28">
-        <v>0.7314000000000001</v>
+        <v>0.7124</v>
       </c>
       <c r="F28">
-        <v>0.034</v>
+        <v>0.0316</v>
       </c>
       <c r="G28">
-        <v>0.0214</v>
+        <v>0.018</v>
       </c>
       <c r="H28">
-        <v>0.0164</v>
+        <v>0.0132</v>
       </c>
       <c r="I28">
-        <v>0.098</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="J28">
-        <v>0.7314000000000001</v>
+        <v>0.7124</v>
       </c>
       <c r="K28">
-        <v>0.7314000000000001</v>
+        <v>0.7124</v>
       </c>
     </row>
     <row r="29">
@@ -1297,31 +1297,31 @@
         <v>5000</v>
       </c>
       <c r="C30">
-        <v>0.0268</v>
+        <v>0.0286</v>
       </c>
       <c r="D30">
-        <v>0.2394</v>
+        <v>0.2326</v>
       </c>
       <c r="E30">
-        <v>0.0266</v>
+        <v>0.0214</v>
       </c>
       <c r="F30">
-        <v>0.0232</v>
+        <v>0.0264</v>
       </c>
       <c r="G30">
-        <v>0.3674</v>
+        <v>0.3724</v>
       </c>
       <c r="H30">
-        <v>0.2744</v>
+        <v>0.2668</v>
       </c>
       <c r="I30">
-        <v>0.07539999999999999</v>
+        <v>0.0746</v>
       </c>
       <c r="J30">
-        <v>0.2937333333333333</v>
+        <v>0.2906</v>
       </c>
       <c r="K30">
-        <v>0.2947818793133958</v>
+        <v>0.2920606264377986</v>
       </c>
     </row>
     <row r="31">
@@ -1332,31 +1332,31 @@
         <v>5000</v>
       </c>
       <c r="C31">
-        <v>0.0372</v>
+        <v>0.05</v>
       </c>
       <c r="D31">
-        <v>0.097</v>
+        <v>0.099</v>
       </c>
       <c r="E31">
-        <v>0.0424</v>
+        <v>0.037</v>
       </c>
       <c r="F31">
-        <v>0.0306</v>
+        <v>0.0364</v>
       </c>
       <c r="G31">
-        <v>0.189</v>
+        <v>0.2042</v>
       </c>
       <c r="H31">
-        <v>0.1198</v>
+        <v>0.1242</v>
       </c>
       <c r="I31">
-        <v>0.0968</v>
+        <v>0.1052</v>
       </c>
       <c r="J31">
-        <v>0.1352666666666667</v>
+        <v>0.1424666666666667</v>
       </c>
       <c r="K31">
-        <v>0.1362048840913113</v>
+        <v>0.1436077508405592</v>
       </c>
     </row>
     <row r="32">
@@ -1393,31 +1393,31 @@
         <v>5000</v>
       </c>
       <c r="C33">
-        <v>0.8274</v>
+        <v>0.8286</v>
       </c>
       <c r="D33">
-        <v>0.0238</v>
+        <v>0.025</v>
       </c>
       <c r="E33">
-        <v>0.8653999999999999</v>
+        <v>0.8618</v>
       </c>
       <c r="F33">
-        <v>0.6634</v>
+        <v>0.6562</v>
       </c>
       <c r="G33">
-        <v>0.0232</v>
+        <v>0.0234</v>
       </c>
       <c r="H33">
-        <v>0.0222</v>
+        <v>0.0272</v>
       </c>
       <c r="I33">
-        <v>0.0678</v>
+        <v>0.0746</v>
       </c>
       <c r="J33">
-        <v>0.7854</v>
+        <v>0.7822</v>
       </c>
       <c r="K33">
-        <v>0.786140594856461</v>
+        <v>0.7828506734902174</v>
       </c>
     </row>
     <row r="34">
@@ -1428,31 +1428,31 @@
         <v>5000</v>
       </c>
       <c r="C34">
-        <v>0.9004</v>
+        <v>0.8962</v>
       </c>
       <c r="D34">
-        <v>0.1138</v>
+        <v>0.1134</v>
       </c>
       <c r="E34">
-        <v>0.9156</v>
+        <v>0.919</v>
       </c>
       <c r="F34">
-        <v>0.7864</v>
+        <v>0.7762</v>
       </c>
       <c r="G34">
-        <v>0.1228</v>
+        <v>0.124</v>
       </c>
       <c r="H34">
-        <v>0.1128</v>
+        <v>0.1258</v>
       </c>
       <c r="I34">
-        <v>0.2368</v>
+        <v>0.2556</v>
       </c>
       <c r="J34">
-        <v>0.8674666666666666</v>
+        <v>0.8638</v>
       </c>
       <c r="K34">
-        <v>0.8677689346347917</v>
+        <v>0.864247047999655</v>
       </c>
     </row>
   </sheetData>

</xml_diff>